<commit_message>
Dancing On My Own (#8): show.yaml aus dem eingefrorenen Code, bridge + outro aus der Tabelle, Strobo-Tails über gate
Szenen und Schemata Part für Part übernommen; bridge (Takt 56) wie der erste Pre-Chorus,
outro (Takt 136) blendet aus; Strobo-Absprünge als SCENE_COLORS + gate statt progStrobo.
Effekt-Katalog: Urteil zu progMatrixRainColor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/DancingOnMyOwn_v1/quelle/struktur.xlsx
+++ b/songs/DancingOnMyOwn_v1/quelle/struktur.xlsx
@@ -541,9 +541,8 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-pause (ab 0:00.000): [SCROLLMATRIX] progBlack(2673, 1); [GITBOARD] progScrollText("Dancing On My Own by Robyn", 15984, 90, getRandomColor(), 2); [sonst] progBlack(5656, 5); [SCROLLMATRIX]
-   Start-MIDI: alle Geräte schwarz</t>
+          <t>progBlack(5656, 5), Farben SCHEME_NEON
+Start-MIDI: alle Geräte schwarz</t>
         </is>
       </c>
       <c r="D6" s="6" t="n"/>
@@ -690,9 +689,8 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-bass (ab 0:05.656): setColorScheme(SCHEME_ICE); scene(SCENE_CALM, 15737, 10, 122);
-   nur Synth-Bass, dunkel und kühl anfangen</t>
+          <t>SCENE_CALM, Farben SCHEME_ICE
+nur Synth-Bass: alle Geräte atmen langsam in Blau, dunkel und kühl</t>
         </is>
       </c>
       <c r="D18" s="6" t="n"/>
@@ -1059,9 +1057,8 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-verse 1 (ab 0:21.393): setColorScheme(SCHEME_ICE); scene(SCENE_VERSE, 15738, 15, 122);
-   Gesang setzt ein, Puls auf allen Geräten, noch kalt</t>
+          <t>SCENE_VERSE, Farben SCHEME_ICE
+Gesang setzt ein: Gitarre und Bass leuchten Zone für Zone im Beat, Lampen mit Lichtschuss pro Beat, auf der Matrix farbiger Regen in Blautönen</t>
         </is>
       </c>
       <c r="D50" s="6" t="n"/>
@@ -1428,9 +1425,9 @@
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-verse 1b (ab 0:37.131): setColorScheme(SCHEME_ROYAL); [ANDRESGIT] progSymmetricVU(15738, 20, 122); [GUITAR] progZoneBeat(15738, 20, 122); [sonst] scene(SCENE_VERSE, 15738, 20, 122);
-   Gitarre steigt ein und bekommt ein eigenes VU, Rest bleibt im Verse-Puls</t>
+          <t>SCENE_VERSE, Farben SCHEME_ROYAL
+ANDRESGIT: progSymmetricVU(15738, 20, 122)
+Gitarre steigt ein und bekommt ein eigenes VU, der Rest bleibt im Verse-Puls, Farben Blau/Violett</t>
         </is>
       </c>
       <c r="D82" s="6" t="n"/>
@@ -1797,9 +1794,8 @@
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-pre-chorus (ab 0:52.869): setColorScheme(SCHEME_SUNSET); scene(SCENE_BUILDUP, 7869, 25, 122);
-   lädt sich über 4 Takte auf und entlädt sich genau in den Chorus</t>
+          <t>SCENE_BUILDUP, Farben SCHEME_SUNSET
+Pre-Chorus: lädt sich über 4 Takte in warmen Farben auf und entlädt sich genau auf den Chorus</t>
         </is>
       </c>
       <c r="D114" s="6" t="n"/>
@@ -1990,9 +1986,8 @@
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-chorus 1 (ab 1:00.738): setColorScheme(SCHEME_NEON); scene(SCENE_DROP, 15737, 30, 122);
-   erster Chorus, volle Energie im Beat</t>
+          <t>SCENE_DROP, Farben SCHEME_NEON
+erster Chorus: volle Energie im Beat in Pink, Türkis und Violett</t>
         </is>
       </c>
       <c r="D130" s="6" t="n"/>
@@ -2359,9 +2354,8 @@
       </c>
       <c r="C162" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-chorus 1b (ab 1:16.475): scene(SCENE_WAVE_LR, 7869, 35, 122);
-   Bühnenbewegung als Variation</t>
+          <t>SCENE_WAVE_LR, Farben SCHEME_NEON
+Blitz läuft auf jedem Beat von links nach rechts über die Bühne</t>
         </is>
       </c>
       <c r="D162" s="6" t="n"/>
@@ -2552,10 +2546,10 @@
       </c>
       <c r="C178" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-hook 1 (ab 1:24.344): scene(SCENE_PINGPONG, 6886, 40, 122);
-   'on my own' springt von Gerät zu Gerät, kurzer Strobo als Absprung in den Stopp
-hook 1 (tail) (ab 1:31.230): progStrobo(983, 45, 75, getRandomCRGB());</t>
+          <t>SCENE_PINGPONG, Farben SCHEME_NEON
+Schluss (2 Beats): SCENE_COLORS, Farben SCHEME_NEON
+   Ausgabe: Tor 4x pro Beat, 50 % hell
+'on my own' springt pro Beat von Gerät zu Gerät; die letzten 2 Beats Strobo im Takt als Absprung in den Stopp</t>
         </is>
       </c>
       <c r="D178" s="6" t="n"/>
@@ -2746,8 +2740,8 @@
       </c>
       <c r="C194" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-stop (ab 1:32.213): progBlack(3935, 50);</t>
+          <t>progBlack(3935, 50), Farben SCHEME_NEON
+Stopp: alles dunkel</t>
         </is>
       </c>
       <c r="D194" s="6" t="n"/>
@@ -2850,9 +2844,8 @@
       </c>
       <c r="C202" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-verse 2 (ab 1:36.148): setColorScheme(SCHEME_ROYAL); scene(SCENE_VERSE, 19672, 55, 122);
-   zurück in den Puls, eine Stufe wärmer als Verse 1</t>
+          <t>SCENE_VERSE, Farben SCHEME_ROYAL
+zurück in den Puls, eine Stufe wärmer als Verse 1 (Blau/Violett), auf der Matrix farbiger Regen</t>
         </is>
       </c>
       <c r="D202" s="6" t="n"/>
@@ -3132,9 +3125,8 @@
       </c>
       <c r="C226" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-verse 2 (ab 1:36.148): setColorScheme(SCHEME_ROYAL); scene(SCENE_VERSE, 19672, 55, 122);
-   zurück in den Puls, eine Stufe wärmer als Verse 1</t>
+          <t>SCENE_BUILDUP, Farben SCHEME_SUNSET
+wie der erste Pre-Chorus: lädt sich über 4 Takte in warmen Farben auf und entlädt sich genau auf den Chorus</t>
         </is>
       </c>
       <c r="D226" s="6" t="n"/>
@@ -3321,8 +3313,8 @@
       </c>
       <c r="C242" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-chorus 2 (ab 1:55.820): scene(SCENE_DROP, 15737, 60, 122);</t>
+          <t>SCENE_DROP, Farben SCHEME_NEON
+zweiter Chorus wie der erste: volle Energie im Beat in Neonfarben</t>
         </is>
       </c>
       <c r="D242" s="6" t="n"/>
@@ -3689,9 +3681,8 @@
       </c>
       <c r="C274" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-chorus 2b (ab 2:11.557): scene(SCENE_WAVE_RL, 7869, 65, 122);
-   Welle diesmal andersrum</t>
+          <t>SCENE_WAVE_RL, Farben SCHEME_NEON
+Blitzwelle diesmal von rechts nach links</t>
         </is>
       </c>
       <c r="D274" s="6" t="n"/>
@@ -3882,8 +3873,8 @@
       </c>
       <c r="C290" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-hook 2 (ab 2:19.426): scene(SCENE_PINGPONG, 7869, 70, 122);</t>
+          <t>SCENE_PINGPONG, Farben SCHEME_NEON
+'on my own' springt pro Beat von Gerät zu Gerät</t>
         </is>
       </c>
       <c r="D290" s="6" t="n"/>
@@ -4074,9 +4065,8 @@
       </c>
       <c r="C306" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-instrumental (ab 2:27.295): setColorScheme(SCHEME_RETRO); scene(SCENE_SOLO_GIT, 15738, 75, 122);
-   Gitarre im Spotlight, rot/weiß/blau wie im Original</t>
+          <t>SCENE_SOLO_GIT, Farben SCHEME_RETRO
+Gitarre im Spotlight, rot/weiß/blau wie im Original</t>
         </is>
       </c>
       <c r="D306" s="6" t="n"/>
@@ -4443,9 +4433,9 @@
       </c>
       <c r="C338" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-bridge (ab 2:43.033): setColorScheme(SCHEME_ICE); [MATRIX] matrixMovieFX(15737, 80, 100, 6); [sonst] scene(SCENE_CALM, 15737, 80, 122);
-   alles zieht sich zurück, Matrix-Film wie im Original</t>
+          <t>SCENE_CALM, Farben SCHEME_ICE
+matrix: matrixMovieFX(15737, 85, 100, 6)
+alles zieht sich zurück und atmet in Blau, auf der Matrix ein dünner Matrix-Regen (6 Spuren) wie im Original</t>
         </is>
       </c>
       <c r="D338" s="6" t="n"/>
@@ -4812,9 +4802,8 @@
       </c>
       <c r="C370" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-corner (ab 2:58.770): progBlack(5902, 85);
-   Stille vor dem Finale</t>
+          <t>progBlack(5902, 90), Farben SCHEME_NEON
+Stille vor dem Finale</t>
         </is>
       </c>
       <c r="D370" s="6" t="n"/>
@@ -4961,9 +4950,8 @@
       </c>
       <c r="C382" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-snare roll (ab 3:04.672): setColorScheme(SCHEME_WHITE); scene(SCENE_BUILDUP, 1967, 90, 122);
-   1 Takt Aufladen, Blast genau auf den Einsatz</t>
+          <t>SCENE_BUILDUP, Farben SCHEME_WHITE
+1 Takt weißes Aufladen, die Explosion fällt genau auf den Einsatz</t>
         </is>
       </c>
       <c r="D382" s="6" t="n"/>
@@ -5022,9 +5010,8 @@
       </c>
       <c r="C386" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-chorus 3 (ab 3:06.639): setColorScheme(SCHEME_FIRE); scene(SCENE_FIRE, 7869, 95, 122);
-   Finale beginnt, Farbwechsel auf Feuer</t>
+          <t>SCENE_FIRE, Farben SCHEME_FIRE
+Finale beginnt: Feuer auf allen Geräten</t>
         </is>
       </c>
       <c r="D386" s="6" t="n"/>
@@ -5215,8 +5202,8 @@
       </c>
       <c r="C402" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-hook 3 (ab 3:14.508): setColorScheme(SCHEME_FIRE); scene(SCENE_WAVE_OUT, 7869, 100, 122);</t>
+          <t>SCENE_WAVE_OUT, Farben SCHEME_FIRE
+Blitz läuft pro Beat von der Mitte nach außen, in Feuerfarben</t>
         </is>
       </c>
       <c r="D402" s="6" t="n"/>
@@ -5407,8 +5394,8 @@
       </c>
       <c r="C418" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-chorus 4 (ab 3:22.377): setColorScheme(SCHEME_SUNSET); scene(SCENE_DROP, 15738, 105, 122);</t>
+          <t>SCENE_DROP, Farben SCHEME_SUNSET
+volle Energie im Beat in Orange, Pink, Violett und Gold</t>
         </is>
       </c>
       <c r="D418" s="6" t="n"/>
@@ -5775,8 +5762,8 @@
       </c>
       <c r="C450" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-chorus 4b (ab 3:38.115): setColorScheme(SCHEME_SUNSET); scene(SCENE_PINGPONG, 7869, 110, 122);</t>
+          <t>SCENE_PINGPONG, Farben SCHEME_SUNSET
+Licht springt pro Beat von Gerät zu Gerät, Sonnenuntergangsfarben</t>
         </is>
       </c>
       <c r="D450" s="6" t="n"/>
@@ -5967,8 +5954,8 @@
       </c>
       <c r="C466" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-hook 4 (ab 3:45.984): setColorScheme(SCHEME_SUNSET); scene(SCENE_WAVE_LR, 7868, 115, 122);</t>
+          <t>SCENE_WAVE_LR, Farben SCHEME_SUNSET
+Blitzwelle von links nach rechts, Sonnenuntergangsfarben</t>
         </is>
       </c>
       <c r="D466" s="6" t="n"/>
@@ -6159,10 +6146,10 @@
       </c>
       <c r="C482" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-hook 5 (ab 3:53.852): setColorScheme(SCHEME_FIRE); scene(SCENE_FIRE, 13771, 120, 122);
-   Höhepunkt, letzter Takt weißer Strobo
-hook 5 (tail) (ab 4:07.623): setColorScheme(SCHEME_FIRE); progStrobo(1967, 125, 65, CRGB::White);</t>
+          <t>SCENE_FIRE, Farben SCHEME_FIRE
+Schluss (4 Beats): SCENE_COLORS, Farben SCHEME_WHITE
+   Ausgabe: Tor 4x pro Beat, 50 % hell
+Höhepunkt: Feuer auf allen Geräten, der letzte Takt weißer Strobo im Takt</t>
         </is>
       </c>
       <c r="D482" s="6" t="n"/>
@@ -6529,9 +6516,8 @@
       </c>
       <c r="C514" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-outro (ab 4:09.590): setColorScheme(SCHEME_SUNSET); scene(SCENE_CALM, 15738, 130, 122);
-   ausatmen</t>
+          <t>SCENE_CALM, Farben SCHEME_SUNSET
+ausatmen: alle Geräte atmen langsam in warmen Farben</t>
         </is>
       </c>
       <c r="D514" s="6" t="n"/>
@@ -6898,8 +6884,8 @@
       </c>
       <c r="C546" s="6" t="inlineStr">
         <is>
-          <t>generierter Code (eingefroren, ohne show.yaml):
-zu dieser Zeit ist der generierte Code schon zu Ende (schwarz, dann Pausen-Loop)</t>
+          <t>SCENE_FADEOUT, Farben SCHEME_SUNSET
+die letzten 2 Takte blenden weich nach Schwarz</t>
         </is>
       </c>
       <c r="D546" s="6" t="n"/>

</xml_diff>